<commit_message>
add today for the start part
</commit_message>
<xml_diff>
--- a/pin2024_cat/SSD_PIN2024.xlsx
+++ b/pin2024_cat/SSD_PIN2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acted-my.sharepoint.com/personal/martina_vit_impact-initiatives_org/Documents/PiN_app_dev/pin2024_cat/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_6AF9E0CFAACBEE72260293B9BFAC01FA80B1BA91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C08E18C9-28B9-4559-8C67-8E70A704BBE1}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_6AF9E0CFAACBEE72260293B9BFAC01FA80B1BA91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F2D1D64-BB69-4815-96FD-B8F010CCBC97}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="host_community" sheetId="1" r:id="rId1"/>
@@ -289,6 +289,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -4606,12 +4607,13 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5940141-1bc9-4c17-b1bc-e50f6b2083d6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4838,19 +4840,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5940141-1bc9-4c17-b1bc-e50f6b2083d6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0B145AD1-2804-49E7-9991-6EA890A5313B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A34D09B0-E945-4CE3-81FD-3E528E7B0F86}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4875,11 +4878,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A34D09B0-E945-4CE3-81FD-3E528E7B0F86}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0B145AD1-2804-49E7-9991-6EA890A5313B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>